<commit_message>
fix: intégration de la relecture critique indépendante
Contenu des PV non inventé, AL-1048 sans examen tracé, P17 nuancé,
scan WEB01 limité à la DMZ, critères G3 uniformes (réalisation 1),
Q05 à 2, Q11 discuté, risques résiduels complets, Kanban à l'état
initial, dépendances début-début, Excel livré avec valeurs calculées.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/livrables/MEDICA-SERVICES_Grille_Audit_SSI_completee.xlsx
+++ b/livrables/MEDICA-SERVICES_Grille_Audit_SSI_completee.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Les environnements contiennent des identifiants patients et des informations de santé. Une altération non détectée peut provoquer des erreurs de prise en charge (P05). Pour un hébergeur d'applications de soins, cette perte de confiance peut être fatale à l'activité.</t>
+          <t>Les environnements contiennent des identifiants patients et des informations de santé. Une altération non détectée peut provoquer des erreurs d'orientation et de prise en charge (P05). L'impact est grave pour l'activité. Aucune pièce ne le décrit comme fatal pour l'entreprise, d'où 2 par cohérence avec Q02 et Q04.</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Portail HTTPS publié sur Internet via WEB01 en DMZ (P03, T02) et interconnexions clients encadrées par contrat (P07). Ouverture externe sous contrôle. La note 3 deviendrait défendable si ces contrôles se révélaient inopérants, la somme passerait alors à 11.</t>
+          <t>Interconnexions clients encadrées par contrat (P07). Le portail est ouvert à des internautes non maîtrisés, mais par une publication unique filtrée (FW-01, FW-08) et un reverse proxy en DMZ (P03, T01, T02). Ouverture externe jugée sous contrôle. La note 3 serait défendable si l'on considère que l'accès public au portail échappe au contrôle de l'organisme. La somme passerait alors à 11 et la cible à 5.</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Niveau 1 étayé par la note d'orientation 2024 approuvée par la DG, des priorités annuelles et un référent (P09). Niveau 2 indéterminé car aucune mesure qualitative n'est produite et le compte rendu semestriel reste oral, sans trace. Niveau 3 non atteint, faute de processus commun documenté (P09). Revue annuelle de la PSSI sans PV depuis deux ans (P17).</t>
+          <t>Niveau 1 étayé par la note d'orientation 2024 approuvée par la DG, des priorités annuelles et un référent (P09). Niveau 2 indéterminé car aucune mesure qualitative n'est documentée et le compte rendu semestriel reste oral, sans trace écrite fournie. Niveau 3 non atteint, faute de processus commun documenté (P09). Revue annuelle de la PSSI sans PV depuis deux ans (P17).</t>
         </is>
       </c>
       <c r="F2" s="10">
@@ -938,7 +938,7 @@
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
-          <t>Tableau de bord qualitatif semestriel et comptes rendus écrits validés par la DG. Preuve : deux PV de revue datés.</t>
+          <t>Tableau de bord qualitatif semestriel et comptes rendus écrits validés par la DG, intégrés au lot A01 (pilote RSSI). Preuve : deux PV de revue datés.</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Besoins identifiés sur certains projets, fiche type, responsable technique, revues planifiées pour les projets majeurs avec compte rendu (P13). Niveau 3 non atteint, la démarche n'est pas globale. La règle FW-17 déclarée provisoire et toujours active (T02) montre que les changements mineurs échappent à la démarche.</t>
+          <t>Besoins identifiés sur certains projets, fiche type, responsable technique désigné, revues planifiées pour les projets majeurs avec compte rendu écrit remonté au responsable (P13). Le compte rendu écrit des revues est retenu comme mesure qualitative. La compétence est retenue, comme pour les autres processus, sur la base d'un rôle désigné chargé de la sécurité, à confirmer en entretien. Niveau 3 non atteint, la démarche n'est pas globale. La règle provisoire FW-17 (T02) l'illustre sans le prouver.</t>
         </is>
       </c>
       <c r="F6" s="10">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Techniciens compétents, comptes rendus d'installation et de validation, suivi régulier avec information de la DSI (P14). La planification est déduite de la préparation et du suivi réguliers, elle reste à confirmer sur pièces. Niveau 3 non atteint. Règles FW-17 et FW-31 sans justification ni validation (T02).</t>
+          <t>Niveau 1 étayé par des déploiements préparés par des techniciens compétents (P14). Comptes rendus d'installation et de validation, suivi régulier et information de la DSI couvrent quatre exigences du niveau 2. Niveau 2 indéterminé car la planification n'est pas démontrée, P14 indiquant seulement que les déploiements sont « souvent préparés ». Règles FW-17 et FW-31 sans justification ni validation (T02).</t>
         </is>
       </c>
       <c r="F7" s="10">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Modèle commun de recette sécurité et revue des règles déployées. Preuve : PV de recette standardisés sur trois déploiements.</t>
+          <t>Plan de déploiement trimestriel des mesures et modèle commun de recette, en régie (pilote DSI). Preuve : plans datés et PV de recette sur trois déploiements.</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Sauvegardes planifiées, comptes rendus hebdomadaires, astreinte, procédure de restauration connue et bilan qualitatif mensuel à la DSI (P15). Niveau 3 non atteint. Fragilités : 2 PV de test sur 9 services (T09), MFA sur 6 comptes privilégiés sur 10 (T04), correctifs en retard sans exception (T06), déclarations contredites (P17).</t>
+          <t>Sauvegardes planifiées, comptes rendus hebdomadaires, astreinte, procédure de restauration connue et bilan qualitatif mensuel à la DSI (P15). Niveau 3 non atteint. Fragilités : 2 PV de test sur 9 services (T09), MFA sur 6 comptes privilégiés sur 10 (T04), correctifs en retard sans exception (T06), déclarations de la DG non démontrées et de la DSI contredites (P17).</t>
         </is>
       </c>
       <c r="F8" s="10">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>APP01 (criticité métier critique) sans correctif critique éditeur (CVSS communiqué 9,8), retard de 74 jours au 12/10/2026, exception non documentée.</t>
+          <t>APP01 (criticité métier critique) sans correctif critique éditeur (CVSS communiqué 9,8, T05). L'hôte affiche 74 jours de retard de correctifs au 12/10/2026, exception non documentée (T06).</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>Non exposé directement à Internet et non exploité pendant l'audit. CVE, version et historique de déploiement absents. Retard déclaratif.</t>
+          <t>Non exposé directement à Internet et non exploité pendant l'audit. Date de publication du correctif critique, CVE, version et historique de déploiement absents. Retard déclaratif.</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>Responsable infrastructures : correctif sous 15 jours ou exception signée avec mesures compensatoires (A09).</t>
+          <t>Responsable infrastructures : correctif sous 15 jours ou exception signée avec mesures compensatoires, traité en tête du lot A09.</t>
         </is>
       </c>
       <c r="I4" s="12" t="inlineStr">
@@ -1392,12 +1392,12 @@
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Usage frauduleux d'un compte dormant non détecté et persistance de privilèges (R01).</t>
+          <t>Usage frauduleux non détecté d'un compte à privilèges et persistance de droits (R01).</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Très élevée : privilège Domain Admin, compte dormant sans MFA, alerte non examinée.</t>
+          <t>Très élevée : privilège Domain Admin, compte sans MFA, aucun examen de l'alerte tracé.</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>L'absence de PV ne prouve pas l'absence de test. Les deux PV ne prouvent pas le RTO de 8 h (P01). Déclaration de la DG contredite (P17).</t>
+          <t>L'absence de PV ne prouve pas l'absence de test. Le contenu des deux PV n'est pas communiqué, le respect du RTO de 8 h n'est donc pas démontré (P01, T09). Déclaration de la DG non démontrée (P17).</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1565,12 +1565,12 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>WEB01 répond sur 80/tcp et 443/tcp, 22/tcp filtré. Le scanner signale TLS 1.0 (CVSS 5,3). La redirection HTTP vers HTTPS est déclarée, non vérifiée.</t>
+          <t>Depuis le point de mesure DMZ, WEB01 répond sur 80/tcp et 443/tcp, 22/tcp filtré. Le scanner signale TLS 1.0 (CVSS 5,3). La redirection HTTP vers HTTPS est déclarée, non vérifiée.</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Validation manuelle absente. Un port ouvert ne prouve pas une faille exploitée.</t>
+          <t>Scan non authentifié depuis la DMZ, aucune vue depuis Internet. Validation manuelle absente. Un port ouvert ne prouve pas une faille exploitée.</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Exploitation web : désactiver TLS 1.0 et 1.1, vérifier la redirection et activer HSTS (A09).</t>
+          <t>Responsable infrastructures : désactiver TLS 1.0 et 1.1, vérifier la redirection et activer HSTS, scan externe de contrôle (A09).</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>4 comptes privilégiés sur 10 sans MFA dont admin-old dormant et admin-presta, RDP direct FW-17, AL-1048 non traitée</t>
+          <t>4 comptes privilégiés sur 10 non enrôlés MFA dont admin-old (dernière activité documentée en 2025, T03) et admin-presta, RDP direct FW-17, AL-1048 fermée sans examen tracé</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>MFA sur 6 comptes sur 10, SIEM avec alertes, bastion pour une partie des accès</t>
+          <t>MFA enrôlé sur 6 comptes sur 10, SIEM avec alertes, bastion pour une partie des accès</t>
         </is>
       </c>
       <c r="G2" s="10" t="n">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Correctif critique manquant depuis 74 jours, aucun SLA, flux WEB01 vers APP01, RDP FW-17</t>
+          <t>Correctif critique manquant (T05), hôte en retard de 74 jours (T06), aucun SLA, flux WEB01 vers APP01, RDP FW-17</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Divulgation de données de santé depuis les partages de fichiers après compromission d'un poste</t>
+          <t>Divulgation de données internes depuis les partages de fichiers après compromission d'un poste, y compris des données de santé si les partages en contiennent (hypothèse)</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>Publication HTTPS sur 443, SSH filtré</t>
+          <t>Publication limitée à 443 et 80 par FW-01 et FW-08, reverse proxy en DMZ</t>
         </is>
       </c>
       <c r="G6" s="10" t="n">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Réduire à faible coût dans A09, sinon accepter temporairement.</t>
+          <t>Réduire à faible coût dans A09. À défaut, acceptation temporaire par la DSI.</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>T+4 mois : méthode, registre consolidé approuvé par la DG, revue trimestrielle</t>
+          <t>T+4 mois : méthode, registre consolidé approuvé par la DG, revue trimestrielle, tableau de bord stratégique semestriel</t>
         </is>
       </c>
       <c r="G2" s="10" t="n">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H2" s="12" t="inlineStr">
         <is>
-          <t>Gérer les risques au niveau 1 (P10). Base de tous les arbitrages R01 à R06.</t>
+          <t>Gérer les risques au niveau 1 (P10). Base de tous les arbitrages R01 à R06. Porte aussi l'étape stratégie (comptes rendus écrits).</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>La mesure quantitative relève du niveau 4, prématurée avec des processus à 1 ou 2. Alternative à A11, non cumulée.</t>
+          <t>La mesure quantitative relève du niveau 4, prématurée avec des processus à 1 ou 2. Alternative à A11, non cumulée. Risque résiduel : pilotage sans indicateurs chiffrés.</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Utile mais moins urgente que R01 et R02. Accompagnement porté en interne par le RSSI.</t>
+          <t>Utile mais moins urgente que R01 et R02. Risque résiduel : adhésion insuffisante aux nouvelles pratiques, suivie par la DG et les managers.</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>C01, C04, C11. R01 et R02. Déclaration P17 contredite.</t>
+          <t>C01, C04, C11. R01 et R02. Déclaration de la DSI contredite par T04.</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>T+4 mois : inventaire authentifié, SLA par criticité, APP01 corrigé, TLS 1.0 retiré, signature SMB</t>
+          <t>APP01 sous 15 jours, puis T+4 mois : inventaire authentifié, SLA par criticité, TLS 1.0 retiré, signature SMB</t>
         </is>
       </c>
       <c r="G10" s="10" t="n">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Recoupe A02 pour le workflow d'alerte. Outil à choisir après stabilisation au niveau 2. Alternative à A06.</t>
+          <t>Recoupe A02 pour le workflow d'alerte. Outil à choisir après stabilisation au niveau 2. Alternative à A06. Risque résiduel : détection limitée sur R01, compensée en partie par A02.</t>
         </is>
       </c>
     </row>

</xml_diff>